<commit_message>
Reporte PDF para el contador y atajos de período al exportar
- src/accounting/pdf.js: resumen por mercado (FIFO), por mes y por exchange, controles, calidad de datos y notas
- GET/POST /api/v1/export/pdf
- Exportar: botones Este mes / Mes anterior / Este año / Año anterior y Reporte PDF
- Ejemplo en examples/ArbiTrack_ejemplo.pdf; pruebas del endpoint

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GyKbiBf481PEtQVoQ9LEzD
</commit_message>
<xml_diff>
--- a/examples/ArbiTrack_ejemplo.xlsx
+++ b/examples/ArbiTrack_ejemplo.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="201">
   <si>
     <t>ArbiTrack P2P — Resumen de resultados</t>
   </si>
@@ -30,7 +30,7 @@
     <t>Período: 2026-09-01 → 2026-09-30 · Horas en America/Lima (UTC−05:00)</t>
   </si>
   <si>
-    <t>Generado: 2026-09-29 20:28:35 · Titular: Ejemplo</t>
+    <t>Generado: 2026-10-20 17:12:47 · Titular: Ejemplo</t>
   </si>
   <si>
     <t>Cada columna es un mercado (par). Importes en la moneda cotizada del par; los pares NO se suman entre sí.</t>
@@ -159,7 +159,7 @@
     <t>Incidencias: errores / advertencias / información</t>
   </si>
   <si>
-    <t>0 / 1 / 1</t>
+    <t>0 / 0 / 1</t>
   </si>
   <si>
     <t>Operaciones contabilizadas</t>
@@ -267,9 +267,6 @@
     <t>p2p_rapido</t>
   </si>
   <si>
-    <t>C-binance_22810000000000000003, C-eldorado_ED-1001</t>
-  </si>
-  <si>
     <t>binance_p2p.csv · fila 3</t>
   </si>
   <si>
@@ -306,24 +303,6 @@
     <t>binance_22810000000000000005</t>
   </si>
   <si>
-    <t>El Dorado</t>
-  </si>
-  <si>
-    <t>ED-1001</t>
-  </si>
-  <si>
-    <t>Rosa</t>
-  </si>
-  <si>
-    <t>C-eldorado_ED-1001</t>
-  </si>
-  <si>
-    <t>eldorado.csv · fila 2</t>
-  </si>
-  <si>
-    <t>eldorado_ED-1001</t>
-  </si>
-  <si>
     <t>22810000000000000006</t>
   </si>
   <si>
@@ -336,33 +315,6 @@
     <t>binance_22810000000000000006</t>
   </si>
   <si>
-    <t>ED-1002</t>
-  </si>
-  <si>
-    <t>Luis</t>
-  </si>
-  <si>
-    <t>C-eldorado_ED-1004</t>
-  </si>
-  <si>
-    <t>eldorado.csv · fila 3</t>
-  </si>
-  <si>
-    <t>eldorado_ED-1002</t>
-  </si>
-  <si>
-    <t>ED-1004</t>
-  </si>
-  <si>
-    <t>Carla</t>
-  </si>
-  <si>
-    <t>eldorado.csv · fila 5</t>
-  </si>
-  <si>
-    <t>eldorado_ED-1004</t>
-  </si>
-  <si>
     <t>Ciclos de arbitraje</t>
   </si>
   <si>
@@ -615,15 +567,6 @@
     <t>estado "cancelado"</t>
   </si>
   <si>
-    <t>ED-1003</t>
-  </si>
-  <si>
-    <t>Pendiente</t>
-  </si>
-  <si>
-    <t>estado "pendiente"</t>
-  </si>
-  <si>
     <t>Incidencias detectadas</t>
   </si>
   <si>
@@ -642,25 +585,13 @@
     <t>Detalle</t>
   </si>
   <si>
-    <t>Advertencia</t>
-  </si>
-  <si>
-    <t>PENDIENTE_ANTIGUA</t>
-  </si>
-  <si>
-    <t>eldorado_ED-1003</t>
-  </si>
-  <si>
-    <t>Sigue pendiente después de 48 h. Vuelva a sincronizar/importar para actualizar su estado.</t>
-  </si>
-  <si>
     <t>Información</t>
   </si>
   <si>
     <t>COMPRA_SIN_VENTA</t>
   </si>
   <si>
-    <t>Quedan 150 USDT de esta compra en inventario (sin venta asociada al cierre del período).</t>
+    <t>Quedan 298.6 USDT de esta compra en inventario (sin venta asociada al cierre del período).</t>
   </si>
   <si>
     <t>METODOLOGÍA DE CÁLCULO — ArbiTrack P2P</t>
@@ -707,7 +638,7 @@
     <numFmt numFmtId="167" formatCode="0.000&quot;%&quot;;[Red]-0.000&quot;%&quot;"/>
     <numFmt numFmtId="168" formatCode="yyyy-mm-dd hh:mm:ss"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -774,11 +705,6 @@
     </font>
     <font>
       <b/>
-      <color rgb="FFB45309"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b/>
       <sz val="13"/>
     </font>
   </fonts>
@@ -832,7 +758,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -872,9 +798,6 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -885,9 +808,8 @@
     <xf numFmtId="3" fontId="11" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1303,7 +1225,7 @@
         <v>10</v>
       </c>
       <c r="C8" s="7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D8" s="7">
         <v>1</v>
@@ -1317,7 +1239,7 @@
         <v>12</v>
       </c>
       <c r="C9" s="8">
-        <v>1200</v>
+        <v>800</v>
       </c>
       <c r="D9" s="8">
         <v>200</v>
@@ -1331,7 +1253,7 @@
         <v>14</v>
       </c>
       <c r="C10" s="9">
-        <v>4446.5</v>
+        <v>2964.5</v>
       </c>
       <c r="D10" s="9">
         <v>200</v>
@@ -1345,7 +1267,7 @@
         <v>14</v>
       </c>
       <c r="C11" s="10">
-        <v>3.70541667</v>
+        <v>3.705625</v>
       </c>
       <c r="D11" s="10">
         <v>1</v>
@@ -1359,7 +1281,7 @@
         <v>10</v>
       </c>
       <c r="C12" s="7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D12" s="7">
         <v>1</v>
@@ -1373,7 +1295,7 @@
         <v>12</v>
       </c>
       <c r="C13" s="8">
-        <v>1048.6</v>
+        <v>500</v>
       </c>
       <c r="D13" s="8">
         <v>200</v>
@@ -1387,7 +1309,7 @@
         <v>14</v>
       </c>
       <c r="C14" s="9">
-        <v>3956.71</v>
+        <v>1886</v>
       </c>
       <c r="D14" s="9">
         <v>202</v>
@@ -1401,7 +1323,7 @@
         <v>14</v>
       </c>
       <c r="C15" s="10">
-        <v>3.77332634</v>
+        <v>3.772</v>
       </c>
       <c r="D15" s="10">
         <v>1.01</v>
@@ -1420,7 +1342,7 @@
         <v>14</v>
       </c>
       <c r="C17" s="9">
-        <v>3956.71</v>
+        <v>1886</v>
       </c>
       <c r="D17" s="9">
         <v>202</v>
@@ -1434,7 +1356,7 @@
         <v>14</v>
       </c>
       <c r="C18" s="9">
-        <v>3885.55</v>
+        <v>1850</v>
       </c>
       <c r="D18" s="9">
         <v>200</v>
@@ -1448,7 +1370,7 @@
         <v>14</v>
       </c>
       <c r="C19" s="12">
-        <v>71.16</v>
+        <v>36</v>
       </c>
       <c r="D19" s="12">
         <v>2</v>
@@ -1462,7 +1384,7 @@
         <v>14</v>
       </c>
       <c r="C20" s="9">
-        <v>1.48</v>
+        <v>0.93</v>
       </c>
       <c r="D20" s="9">
         <v>0</v>
@@ -1490,7 +1412,7 @@
         <v>14</v>
       </c>
       <c r="C22" s="12">
-        <v>61.46</v>
+        <v>26.85</v>
       </c>
       <c r="D22" s="12">
         <v>2</v>
@@ -1504,7 +1426,7 @@
         <v>28</v>
       </c>
       <c r="C23" s="13">
-        <v>1.5818</v>
+        <v>1.4516</v>
       </c>
       <c r="D23" s="13">
         <v>1</v>
@@ -1518,7 +1440,7 @@
         <v>10</v>
       </c>
       <c r="C24" s="7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D24" s="7">
         <v>1</v>
@@ -1565,7 +1487,7 @@
         <v>12</v>
       </c>
       <c r="C28" s="8">
-        <v>150</v>
+        <v>298.6</v>
       </c>
       <c r="D28" s="8">
         <v>0</v>
@@ -1579,7 +1501,7 @@
         <v>14</v>
       </c>
       <c r="C29" s="9">
-        <v>555.75</v>
+        <v>1109.85</v>
       </c>
       <c r="D29" s="9">
         <v>0</v>
@@ -1593,7 +1515,7 @@
         <v>14</v>
       </c>
       <c r="C30" s="10">
-        <v>3.705</v>
+        <v>3.71685843</v>
       </c>
       <c r="D30" s="10">
         <v>0</v>
@@ -1626,7 +1548,7 @@
         <v>14</v>
       </c>
       <c r="C33" s="9">
-        <v>-494.29</v>
+        <v>-1083</v>
       </c>
       <c r="D33" s="9">
         <v>2</v>
@@ -1640,7 +1562,7 @@
         <v>14</v>
       </c>
       <c r="C34" s="9">
-        <v>555.75</v>
+        <v>1109.85</v>
       </c>
       <c r="D34" s="9">
         <v>0</v>
@@ -1665,7 +1587,7 @@
         <v>41</v>
       </c>
       <c r="C37">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -1673,7 +1595,7 @@
         <v>42</v>
       </c>
       <c r="C38">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -1681,7 +1603,7 @@
         <v>43</v>
       </c>
       <c r="C39">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -1713,7 +1635,7 @@
     <tabColor rgb="FF94A3B8"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -1731,7 +1653,7 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>187</v>
+        <v>171</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1763,7 +1685,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>188</v>
+        <v>172</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -1779,7 +1701,7 @@
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>173</v>
+        <v>157</v>
       </c>
       <c r="B5" s="15" t="s">
         <v>49</v>
@@ -1797,22 +1719,22 @@
         <v>53</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="H5" s="15" t="s">
         <v>55</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="J5" s="15" t="s">
         <v>60</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>191</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -1823,13 +1745,13 @@
         <v>68</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>192</v>
+        <v>176</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>193</v>
+        <v>177</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F6" s="17" t="s">
         <v>6</v>
@@ -1844,55 +1766,17 @@
         <v>376.5</v>
       </c>
       <c r="J6" s="17" t="s">
-        <v>194</v>
+        <v>178</v>
       </c>
       <c r="K6" s="17" t="s">
-        <v>195</v>
+        <v>179</v>
       </c>
       <c r="L6" s="17" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" s="22">
-        <v>46280.45833333333</v>
-      </c>
-      <c r="B7" s="23" t="s">
-        <v>94</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>197</v>
-      </c>
-      <c r="D7" s="23" t="s">
-        <v>96</v>
-      </c>
-      <c r="E7" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="F7" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="G7" s="25">
-        <v>250</v>
-      </c>
-      <c r="H7" s="26">
-        <v>3.77</v>
-      </c>
-      <c r="I7" s="27">
-        <v>942.5</v>
-      </c>
-      <c r="J7" s="23" t="s">
-        <v>198</v>
-      </c>
-      <c r="K7" s="23" t="s">
-        <v>198</v>
-      </c>
-      <c r="L7" s="23" t="s">
-        <v>199</v>
+        <v>180</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:L7"/>
+  <autoFilter ref="A5:L6"/>
   <mergeCells count="3">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
@@ -1912,7 +1796,7 @@
     <tabColor rgb="FFB45309"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1926,7 +1810,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>200</v>
+        <v>181</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1950,7 +1834,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>201</v>
+        <v>182</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -1962,13 +1846,13 @@
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>202</v>
+        <v>183</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>203</v>
+        <v>184</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>173</v>
+        <v>157</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>53</v>
@@ -1980,66 +1864,40 @@
         <v>50</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>204</v>
+        <v>185</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>205</v>
+        <v>186</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="40" t="s">
-        <v>206</v>
+      <c r="A6" s="39" t="s">
+        <v>187</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>207</v>
+        <v>188</v>
       </c>
       <c r="C6" s="16">
-        <v>46280.45833333333</v>
+        <v>46267.41887731482</v>
       </c>
       <c r="D6" s="17" t="s">
         <v>6</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>94</v>
+        <v>68</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>197</v>
+        <v>79</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>208</v>
+        <v>82</v>
       </c>
       <c r="H6" s="17" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="41" t="s">
-        <v>210</v>
-      </c>
-      <c r="B7" s="23" t="s">
-        <v>211</v>
-      </c>
-      <c r="C7" s="22">
-        <v>46280.375</v>
-      </c>
-      <c r="D7" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="E7" s="23" t="s">
-        <v>94</v>
-      </c>
-      <c r="F7" s="23" t="s">
-        <v>104</v>
-      </c>
-      <c r="G7" s="23" t="s">
-        <v>108</v>
-      </c>
-      <c r="H7" s="23" t="s">
-        <v>212</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:H7"/>
+  <autoFilter ref="A5:H6"/>
   <mergeCells count="3">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
@@ -2065,63 +1923,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="42" t="s">
-        <v>213</v>
+      <c r="A1" s="40" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="41" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="43" t="s">
-        <v>214</v>
+      <c r="A3" s="41" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="43" t="s">
-        <v>215</v>
+      <c r="A4" s="41" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="43" t="s">
-        <v>216</v>
+      <c r="A5" s="41" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="43" t="s">
-        <v>217</v>
+      <c r="A6" s="41" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="43" t="s">
-        <v>218</v>
+      <c r="A7" s="41" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="43" t="s">
-        <v>219</v>
+      <c r="A8" s="41" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="43" t="s">
-        <v>220</v>
+      <c r="A9" s="41" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="43" t="s">
-        <v>221</v>
+      <c r="A10" s="41" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="43" t="s">
-        <v>222</v>
+      <c r="A11" s="41" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="43" t="s">
-        <v>223</v>
+      <c r="A12" s="41" t="s">
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -2139,7 +1997,7 @@
     <tabColor rgb="FF2563EB"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T13"/>
+  <dimension ref="A1:T10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -2394,7 +2252,7 @@
         <v>73</v>
       </c>
       <c r="N7" s="23" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="O7" s="27"/>
       <c r="P7" s="27"/>
@@ -2405,10 +2263,10 @@
         <v>76</v>
       </c>
       <c r="S7" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="T7" s="23" t="s">
         <v>82</v>
-      </c>
-      <c r="T7" s="23" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
@@ -2419,13 +2277,13 @@
         <v>68</v>
       </c>
       <c r="C8" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="D8" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="D8" s="17" t="s">
+      <c r="E8" s="28" t="s">
         <v>85</v>
-      </c>
-      <c r="E8" s="28" t="s">
-        <v>86</v>
       </c>
       <c r="F8" s="17" t="s">
         <v>6</v>
@@ -2467,10 +2325,10 @@
         <v>76</v>
       </c>
       <c r="S8" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="T8" s="17" t="s">
         <v>87</v>
-      </c>
-      <c r="T8" s="17" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
@@ -2481,10 +2339,10 @@
         <v>68</v>
       </c>
       <c r="C9" s="23" t="s">
+        <v>88</v>
+      </c>
+      <c r="D9" s="23" t="s">
         <v>89</v>
-      </c>
-      <c r="D9" s="23" t="s">
-        <v>90</v>
       </c>
       <c r="E9" s="24" t="s">
         <v>71</v>
@@ -2514,7 +2372,7 @@
         <v>73</v>
       </c>
       <c r="N9" s="23" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="O9" s="27"/>
       <c r="P9" s="27"/>
@@ -2525,39 +2383,39 @@
         <v>76</v>
       </c>
       <c r="S9" s="23" t="s">
+        <v>91</v>
+      </c>
+      <c r="T9" s="23" t="s">
         <v>92</v>
-      </c>
-      <c r="T9" s="23" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="16">
-        <v>46268.76527777778</v>
+        <v>46269.5</v>
       </c>
       <c r="B10" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="D10" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="C10" s="17" t="s">
-        <v>95</v>
-      </c>
-      <c r="D10" s="17" t="s">
-        <v>96</v>
-      </c>
       <c r="E10" s="28" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F10" s="17" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G10" s="19">
-        <v>298.6</v>
+        <v>200</v>
       </c>
       <c r="H10" s="20">
-        <v>3.78</v>
+        <v>1.01</v>
       </c>
       <c r="I10" s="21">
-        <v>1128.71</v>
+        <v>202</v>
       </c>
       <c r="J10" s="19">
         <v>0</v>
@@ -2572,13 +2430,13 @@
         <v>73</v>
       </c>
       <c r="N10" s="17" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="O10" s="21">
-        <v>19.41</v>
+        <v>2</v>
       </c>
       <c r="P10" s="21">
-        <v>18.86</v>
+        <v>2</v>
       </c>
       <c r="Q10" s="17" t="s">
         <v>75</v>
@@ -2587,196 +2445,14 @@
         <v>76</v>
       </c>
       <c r="S10" s="17" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="T10" s="17" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A11" s="22">
-        <v>46269.5</v>
-      </c>
-      <c r="B11" s="23" t="s">
-        <v>68</v>
-      </c>
-      <c r="C11" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="D11" s="23" t="s">
-        <v>101</v>
-      </c>
-      <c r="E11" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="F11" s="23" t="s">
-        <v>7</v>
-      </c>
-      <c r="G11" s="25">
-        <v>200</v>
-      </c>
-      <c r="H11" s="26">
-        <v>1.01</v>
-      </c>
-      <c r="I11" s="27">
-        <v>202</v>
-      </c>
-      <c r="J11" s="25">
-        <v>0</v>
-      </c>
-      <c r="K11" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="L11" s="27">
-        <v>0</v>
-      </c>
-      <c r="M11" s="23" t="s">
-        <v>73</v>
-      </c>
-      <c r="N11" s="23" t="s">
-        <v>91</v>
-      </c>
-      <c r="O11" s="27">
-        <v>2</v>
-      </c>
-      <c r="P11" s="27">
-        <v>2</v>
-      </c>
-      <c r="Q11" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="R11" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="S11" s="23" t="s">
-        <v>102</v>
-      </c>
-      <c r="T11" s="23" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A12" s="16">
-        <v>46280.375</v>
-      </c>
-      <c r="B12" s="17" t="s">
-        <v>94</v>
-      </c>
-      <c r="C12" s="17" t="s">
-        <v>104</v>
-      </c>
-      <c r="D12" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="E12" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="F12" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="G12" s="19">
-        <v>400</v>
-      </c>
-      <c r="H12" s="20">
-        <v>3.705</v>
-      </c>
-      <c r="I12" s="21">
-        <v>1482</v>
-      </c>
-      <c r="J12" s="19">
-        <v>0</v>
-      </c>
-      <c r="K12" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="L12" s="21">
-        <v>0</v>
-      </c>
-      <c r="M12" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="N12" s="17" t="s">
-        <v>106</v>
-      </c>
-      <c r="O12" s="21"/>
-      <c r="P12" s="21"/>
-      <c r="Q12" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="R12" s="17" t="s">
-        <v>76</v>
-      </c>
-      <c r="S12" s="17" t="s">
-        <v>107</v>
-      </c>
-      <c r="T12" s="17" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A13" s="22">
-        <v>46281.4375</v>
-      </c>
-      <c r="B13" s="23" t="s">
-        <v>94</v>
-      </c>
-      <c r="C13" s="23" t="s">
-        <v>109</v>
-      </c>
-      <c r="D13" s="23" t="s">
-        <v>110</v>
-      </c>
-      <c r="E13" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="F13" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="G13" s="25">
-        <v>250</v>
-      </c>
-      <c r="H13" s="26">
-        <v>3.768</v>
-      </c>
-      <c r="I13" s="27">
-        <v>942</v>
-      </c>
-      <c r="J13" s="25">
-        <v>0</v>
-      </c>
-      <c r="K13" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="L13" s="27">
-        <v>0</v>
-      </c>
-      <c r="M13" s="23" t="s">
-        <v>73</v>
-      </c>
-      <c r="N13" s="23" t="s">
-        <v>106</v>
-      </c>
-      <c r="O13" s="27">
-        <v>15.75</v>
-      </c>
-      <c r="P13" s="27">
-        <v>15.75</v>
-      </c>
-      <c r="Q13" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="R13" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="S13" s="23" t="s">
-        <v>111</v>
-      </c>
-      <c r="T13" s="23" t="s">
-        <v>112</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:T13"/>
+  <autoFilter ref="A5:T10"/>
   <mergeCells count="3">
     <mergeCell ref="A1:T1"/>
     <mergeCell ref="A2:T2"/>
@@ -2796,7 +2472,7 @@
     <tabColor rgb="FF7C3AED"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U10"/>
+  <dimension ref="A1:U8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -2818,7 +2494,7 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2868,7 +2544,7 @@
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -2893,7 +2569,7 @@
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -2930,55 +2606,55 @@
         <v>60</v>
       </c>
       <c r="E6" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="F6" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="G6" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="I6" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="J6" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="K6" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="L6" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="M6" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="N6" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="O6" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="P6" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="Q6" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="R6" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="S6" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="T6" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="U6" s="15" t="s">
         <v>116</v>
-      </c>
-      <c r="F6" s="15" t="s">
-        <v>117</v>
-      </c>
-      <c r="G6" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="H6" s="15" t="s">
-        <v>119</v>
-      </c>
-      <c r="I6" s="15" t="s">
-        <v>120</v>
-      </c>
-      <c r="J6" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="K6" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="L6" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="M6" s="15" t="s">
-        <v>124</v>
-      </c>
-      <c r="N6" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="O6" s="15" t="s">
-        <v>126</v>
-      </c>
-      <c r="P6" s="15" t="s">
-        <v>127</v>
-      </c>
-      <c r="Q6" s="15" t="s">
-        <v>128</v>
-      </c>
-      <c r="R6" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="S6" s="15" t="s">
-        <v>130</v>
-      </c>
-      <c r="T6" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="U6" s="15" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
@@ -2986,13 +2662,13 @@
         <v>74</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="C7" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="30" t="s">
-        <v>134</v>
+      <c r="D7" s="29" t="s">
+        <v>118</v>
       </c>
       <c r="E7" s="16">
         <v>46267.3837962963</v>
@@ -3030,10 +2706,10 @@
       <c r="P7" s="21">
         <v>0</v>
       </c>
-      <c r="Q7" s="31">
+      <c r="Q7" s="30">
         <v>35.07</v>
       </c>
-      <c r="R7" s="32">
+      <c r="R7" s="31">
         <v>1.8957</v>
       </c>
       <c r="S7" s="21">
@@ -3041,212 +2717,80 @@
         <v>35.07</v>
       </c>
       <c r="T7" s="17" t="s">
-        <v>135</v>
+        <v>119</v>
       </c>
       <c r="U7" s="17" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" s="23" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" s="33" t="s">
-        <v>134</v>
+        <v>7</v>
+      </c>
+      <c r="D8" s="32" t="s">
+        <v>118</v>
       </c>
       <c r="E8" s="22">
-        <v>46267.41887731482</v>
+        <v>46268.5</v>
       </c>
       <c r="F8" s="22">
-        <v>46268.76527777778</v>
+        <v>46269.5</v>
       </c>
       <c r="G8" s="23" t="s">
         <v>68</v>
       </c>
       <c r="H8" s="23" t="s">
-        <v>94</v>
+        <v>68</v>
       </c>
       <c r="I8" s="25">
-        <v>298.6</v>
+        <v>200</v>
       </c>
       <c r="J8" s="26">
-        <v>3.715</v>
+        <v>1</v>
       </c>
       <c r="K8" s="26">
-        <v>3.78</v>
+        <v>1.01</v>
       </c>
       <c r="L8" s="27">
-        <v>1128.71</v>
+        <v>202</v>
       </c>
       <c r="M8" s="27">
-        <v>1109.3</v>
+        <v>200</v>
       </c>
       <c r="N8" s="27">
-        <v>19.41</v>
+        <v>2</v>
       </c>
       <c r="O8" s="27">
-        <v>0.55</v>
+        <v>0</v>
       </c>
       <c r="P8" s="27">
         <v>0</v>
       </c>
-      <c r="Q8" s="34">
-        <v>18.86</v>
-      </c>
-      <c r="R8" s="35">
-        <v>1.6998</v>
+      <c r="Q8" s="33">
+        <v>2</v>
+      </c>
+      <c r="R8" s="34">
+        <v>1</v>
       </c>
       <c r="S8" s="27">
         <f>SUMIFS($Q$7:Q8,$C$7:C8,C8)</f>
-        <v>53.93</v>
+        <v>2</v>
       </c>
       <c r="T8" s="23" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="U8" s="23" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
-        <v>91</v>
-      </c>
-      <c r="B9" s="17" t="s">
-        <v>133</v>
-      </c>
-      <c r="C9" s="17" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="30" t="s">
-        <v>134</v>
-      </c>
-      <c r="E9" s="16">
-        <v>46268.5</v>
-      </c>
-      <c r="F9" s="16">
-        <v>46269.5</v>
-      </c>
-      <c r="G9" s="17" t="s">
-        <v>68</v>
-      </c>
-      <c r="H9" s="17" t="s">
-        <v>68</v>
-      </c>
-      <c r="I9" s="19">
-        <v>200</v>
-      </c>
-      <c r="J9" s="20">
-        <v>1</v>
-      </c>
-      <c r="K9" s="20">
-        <v>1.01</v>
-      </c>
-      <c r="L9" s="21">
-        <v>202</v>
-      </c>
-      <c r="M9" s="21">
-        <v>200</v>
-      </c>
-      <c r="N9" s="21">
-        <v>2</v>
-      </c>
-      <c r="O9" s="21">
-        <v>0</v>
-      </c>
-      <c r="P9" s="21">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="31">
-        <v>2</v>
-      </c>
-      <c r="R9" s="32">
-        <v>1</v>
-      </c>
-      <c r="S9" s="21">
-        <f>SUMIFS($Q$7:Q9,$C$7:C9,C9)</f>
-        <v>2</v>
-      </c>
-      <c r="T9" s="17" t="s">
-        <v>93</v>
-      </c>
-      <c r="U9" s="17" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A10" s="23" t="s">
-        <v>106</v>
-      </c>
-      <c r="B10" s="23" t="s">
-        <v>133</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="D10" s="33" t="s">
-        <v>134</v>
-      </c>
-      <c r="E10" s="22">
-        <v>46280.375</v>
-      </c>
-      <c r="F10" s="22">
-        <v>46281.4375</v>
-      </c>
-      <c r="G10" s="23" t="s">
-        <v>94</v>
-      </c>
-      <c r="H10" s="23" t="s">
-        <v>94</v>
-      </c>
-      <c r="I10" s="25">
-        <v>250</v>
-      </c>
-      <c r="J10" s="26">
-        <v>3.705</v>
-      </c>
-      <c r="K10" s="26">
-        <v>3.768</v>
-      </c>
-      <c r="L10" s="27">
-        <v>942</v>
-      </c>
-      <c r="M10" s="27">
-        <v>926.25</v>
-      </c>
-      <c r="N10" s="27">
-        <v>15.75</v>
-      </c>
-      <c r="O10" s="27">
-        <v>0</v>
-      </c>
-      <c r="P10" s="27">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="34">
-        <v>15.75</v>
-      </c>
-      <c r="R10" s="35">
-        <v>1.7004</v>
-      </c>
-      <c r="S10" s="27">
-        <f>SUMIFS($Q$7:Q10,$C$7:C10,C10)</f>
-        <v>69.68</v>
-      </c>
-      <c r="T10" s="23" t="s">
-        <v>108</v>
-      </c>
-      <c r="U10" s="23" t="s">
-        <v>112</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:U10"/>
+  <autoFilter ref="A6:U8"/>
   <mergeCells count="4">
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="A2:U2"/>
@@ -3267,7 +2811,7 @@
     <tabColor rgb="FF64748B"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -3286,7 +2830,7 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3318,7 +2862,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>137</v>
+        <v>121</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -3340,37 +2884,37 @@
         <v>53</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>138</v>
+        <v>122</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>139</v>
+        <v>123</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>140</v>
+        <v>124</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>141</v>
+        <v>125</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>142</v>
+        <v>126</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>143</v>
+        <v>127</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>144</v>
+        <v>128</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>145</v>
+        <v>129</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>146</v>
+        <v>130</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>147</v>
+        <v>131</v>
       </c>
       <c r="M5" s="15" t="s">
-        <v>148</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
@@ -3381,10 +2925,10 @@
         <v>6</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>149</v>
+        <v>133</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E6" s="16">
         <v>46267.56946759259</v>
@@ -3422,10 +2966,10 @@
         <v>6</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>149</v>
+        <v>133</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E7" s="22">
         <v>46267.56946759259</v>
@@ -3434,7 +2978,7 @@
         <v>68</v>
       </c>
       <c r="G7" s="23" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H7" s="22">
         <v>46267.41887731482</v>
@@ -3457,129 +3001,47 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>149</v>
+        <v>133</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="E8" s="16">
-        <v>46268.76527777778</v>
+        <v>46269.5</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>94</v>
+        <v>68</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="H8" s="16">
-        <v>46267.41887731482</v>
+        <v>46268.5</v>
       </c>
       <c r="I8" s="17" t="s">
         <v>68</v>
       </c>
       <c r="J8" s="19">
-        <v>298.6</v>
+        <v>200</v>
       </c>
       <c r="K8" s="20">
-        <v>3.715</v>
+        <v>1</v>
       </c>
       <c r="L8" s="21">
-        <v>1109.299</v>
+        <v>200</v>
       </c>
       <c r="M8" s="21">
-        <v>0.55492696</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="23" t="s">
-        <v>106</v>
-      </c>
-      <c r="B9" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>149</v>
-      </c>
-      <c r="D9" s="23" t="s">
-        <v>112</v>
-      </c>
-      <c r="E9" s="22">
-        <v>46281.4375</v>
-      </c>
-      <c r="F9" s="23" t="s">
-        <v>94</v>
-      </c>
-      <c r="G9" s="23" t="s">
-        <v>108</v>
-      </c>
-      <c r="H9" s="22">
-        <v>46280.375</v>
-      </c>
-      <c r="I9" s="23" t="s">
-        <v>94</v>
-      </c>
-      <c r="J9" s="25">
-        <v>250</v>
-      </c>
-      <c r="K9" s="26">
-        <v>3.705</v>
-      </c>
-      <c r="L9" s="27">
-        <v>926.25</v>
-      </c>
-      <c r="M9" s="27">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" s="17" t="s">
-        <v>91</v>
-      </c>
-      <c r="B10" s="17" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>149</v>
-      </c>
-      <c r="D10" s="17" t="s">
-        <v>103</v>
-      </c>
-      <c r="E10" s="16">
-        <v>46269.5</v>
-      </c>
-      <c r="F10" s="17" t="s">
-        <v>68</v>
-      </c>
-      <c r="G10" s="17" t="s">
-        <v>93</v>
-      </c>
-      <c r="H10" s="16">
-        <v>46268.5</v>
-      </c>
-      <c r="I10" s="17" t="s">
-        <v>68</v>
-      </c>
-      <c r="J10" s="19">
-        <v>200</v>
-      </c>
-      <c r="K10" s="20">
-        <v>1</v>
-      </c>
-      <c r="L10" s="21">
-        <v>200</v>
-      </c>
-      <c r="M10" s="21">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A5:M10"/>
+  <autoFilter ref="A5:M8"/>
   <mergeCells count="3">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
@@ -3613,7 +3075,7 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>150</v>
+        <v>134</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3645,7 +3107,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>151</v>
+        <v>135</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -3664,37 +3126,37 @@
         <v>53</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>152</v>
+        <v>136</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>153</v>
+        <v>137</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>11</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>154</v>
+        <v>138</v>
       </c>
       <c r="F5" s="15" t="s">
         <v>17</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>155</v>
+        <v>139</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>156</v>
+        <v>140</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>128</v>
+        <v>112</v>
       </c>
       <c r="L5" s="15" t="s">
-        <v>157</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -3705,39 +3167,39 @@
         <v>72</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>158</v>
+        <v>142</v>
       </c>
       <c r="D6" s="19">
-        <f>SUMIFS(Operaciones!$G$6:$G$13,Operaciones!$F$6:$F$13,"USDT/PEN",Operaciones!$E$6:$E$13,"Compra")</f>
-        <v>1200</v>
+        <f>SUMIFS(Operaciones!$G$6:$G$10,Operaciones!$F$6:$F$10,"USDT/PEN",Operaciones!$E$6:$E$10,"Compra")</f>
+        <v>800</v>
       </c>
       <c r="E6" s="21">
-        <f>SUMIFS(Operaciones!$I$6:$I$13,Operaciones!$F$6:$F$13,"USDT/PEN",Operaciones!$E$6:$E$13,"Compra")</f>
-        <v>4446.5</v>
+        <f>SUMIFS(Operaciones!$I$6:$I$10,Operaciones!$F$6:$F$10,"USDT/PEN",Operaciones!$E$6:$E$10,"Compra")</f>
+        <v>2964.5</v>
       </c>
       <c r="F6" s="19">
-        <f>SUMIFS(Operaciones!$G$6:$G$13,Operaciones!$F$6:$F$13,"USDT/PEN",Operaciones!$E$6:$E$13,"Venta")</f>
-        <v>1048.6</v>
+        <f>SUMIFS(Operaciones!$G$6:$G$10,Operaciones!$F$6:$F$10,"USDT/PEN",Operaciones!$E$6:$E$10,"Venta")</f>
+        <v>500</v>
       </c>
       <c r="G6" s="21">
-        <f>SUMIFS(Operaciones!$I$6:$I$13,Operaciones!$F$6:$F$13,"USDT/PEN",Operaciones!$E$6:$E$13,"Venta")</f>
-        <v>3956.71</v>
+        <f>SUMIFS(Operaciones!$I$6:$I$10,Operaciones!$F$6:$F$10,"USDT/PEN",Operaciones!$E$6:$E$10,"Venta")</f>
+        <v>1886</v>
       </c>
       <c r="H6" s="21">
-        <f>SUMIFS(Operaciones!$L$6:$L$13,Operaciones!$F$6:$F$13,"USDT/PEN")</f>
+        <f>SUMIFS(Operaciones!$L$6:$L$10,Operaciones!$F$6:$F$10,"USDT/PEN")</f>
         <v>1.48</v>
       </c>
       <c r="I6" s="21">
-        <v>71.16</v>
+        <v>36</v>
       </c>
       <c r="J6" s="21">
         <v>8.22</v>
       </c>
-      <c r="K6" s="31">
-        <v>61.46</v>
+      <c r="K6" s="30">
+        <v>26.85</v>
       </c>
       <c r="L6" s="19">
-        <v>150</v>
+        <v>298.6</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -3748,26 +3210,26 @@
         <v>72</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
       <c r="D7" s="25">
-        <f>SUMIFS(Operaciones!$G$6:$G$13,Operaciones!$F$6:$F$13,"USDT/USD",Operaciones!$E$6:$E$13,"Compra")</f>
+        <f>SUMIFS(Operaciones!$G$6:$G$10,Operaciones!$F$6:$F$10,"USDT/USD",Operaciones!$E$6:$E$10,"Compra")</f>
         <v>200</v>
       </c>
       <c r="E7" s="27">
-        <f>SUMIFS(Operaciones!$I$6:$I$13,Operaciones!$F$6:$F$13,"USDT/USD",Operaciones!$E$6:$E$13,"Compra")</f>
+        <f>SUMIFS(Operaciones!$I$6:$I$10,Operaciones!$F$6:$F$10,"USDT/USD",Operaciones!$E$6:$E$10,"Compra")</f>
         <v>200</v>
       </c>
       <c r="F7" s="25">
-        <f>SUMIFS(Operaciones!$G$6:$G$13,Operaciones!$F$6:$F$13,"USDT/USD",Operaciones!$E$6:$E$13,"Venta")</f>
+        <f>SUMIFS(Operaciones!$G$6:$G$10,Operaciones!$F$6:$F$10,"USDT/USD",Operaciones!$E$6:$E$10,"Venta")</f>
         <v>200</v>
       </c>
       <c r="G7" s="27">
-        <f>SUMIFS(Operaciones!$I$6:$I$13,Operaciones!$F$6:$F$13,"USDT/USD",Operaciones!$E$6:$E$13,"Venta")</f>
+        <f>SUMIFS(Operaciones!$I$6:$I$10,Operaciones!$F$6:$F$10,"USDT/USD",Operaciones!$E$6:$E$10,"Venta")</f>
         <v>202</v>
       </c>
       <c r="H7" s="27">
-        <f>SUMIFS(Operaciones!$L$6:$L$13,Operaciones!$F$6:$F$13,"USDT/USD")</f>
+        <f>SUMIFS(Operaciones!$L$6:$L$10,Operaciones!$F$6:$F$10,"USDT/USD")</f>
         <v>0</v>
       </c>
       <c r="I7" s="27">
@@ -3776,7 +3238,7 @@
       <c r="J7" s="27">
         <v>0</v>
       </c>
-      <c r="K7" s="34">
+      <c r="K7" s="33">
         <v>2</v>
       </c>
       <c r="L7" s="25">
@@ -3804,7 +3266,7 @@
     <tabColor rgb="FF14B8A6"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -3819,7 +3281,7 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3851,7 +3313,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>161</v>
+        <v>145</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -3873,31 +3335,31 @@
         <v>49</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>162</v>
+        <v>146</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>11</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>154</v>
+        <v>138</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>163</v>
+        <v>147</v>
       </c>
       <c r="G5" s="15" t="s">
         <v>17</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>155</v>
+        <v>139</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>156</v>
+        <v>140</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>164</v>
+        <v>148</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>165</v>
+        <v>149</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -3907,7 +3369,7 @@
       <c r="B6" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="C6" s="36">
+      <c r="C6" s="35">
         <v>2</v>
       </c>
       <c r="D6" s="19">
@@ -3916,7 +3378,7 @@
       <c r="E6" s="21">
         <v>2964.5</v>
       </c>
-      <c r="F6" s="36">
+      <c r="F6" s="35">
         <v>1</v>
       </c>
       <c r="G6" s="19">
@@ -3931,82 +3393,47 @@
       <c r="J6" s="21">
         <v>36</v>
       </c>
-      <c r="K6" s="31">
+      <c r="K6" s="30">
         <v>35.07</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="23" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>94</v>
-      </c>
-      <c r="C7" s="37">
+        <v>68</v>
+      </c>
+      <c r="C7" s="36">
         <v>1</v>
       </c>
       <c r="D7" s="25">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="E7" s="27">
-        <v>1482</v>
-      </c>
-      <c r="F7" s="37">
-        <v>2</v>
+        <v>200</v>
+      </c>
+      <c r="F7" s="36">
+        <v>1</v>
       </c>
       <c r="G7" s="25">
-        <v>548.6</v>
+        <v>200</v>
       </c>
       <c r="H7" s="27">
-        <v>2070.71</v>
+        <v>202</v>
       </c>
       <c r="I7" s="27">
         <v>0</v>
       </c>
       <c r="J7" s="27">
-        <v>35.16</v>
-      </c>
-      <c r="K7" s="34">
-        <v>34.61</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="17" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="17" t="s">
-        <v>68</v>
-      </c>
-      <c r="C8" s="36">
-        <v>1</v>
-      </c>
-      <c r="D8" s="19">
-        <v>200</v>
-      </c>
-      <c r="E8" s="21">
-        <v>200</v>
-      </c>
-      <c r="F8" s="36">
-        <v>1</v>
-      </c>
-      <c r="G8" s="19">
-        <v>200</v>
-      </c>
-      <c r="H8" s="21">
-        <v>202</v>
-      </c>
-      <c r="I8" s="21">
-        <v>0</v>
-      </c>
-      <c r="J8" s="21">
         <v>2</v>
       </c>
-      <c r="K8" s="31">
+      <c r="K7" s="33">
         <v>2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:K8"/>
+  <autoFilter ref="A5:K7"/>
   <mergeCells count="3">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
@@ -4040,7 +3467,7 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>166</v>
+        <v>150</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4066,7 +3493,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>167</v>
+        <v>151</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -4082,28 +3509,28 @@
         <v>53</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>168</v>
+        <v>152</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>169</v>
+        <v>153</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>123</v>
+        <v>107</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>128</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -4111,28 +3538,28 @@
         <v>6</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>170</v>
-      </c>
-      <c r="C6" s="36">
-        <v>3</v>
+        <v>154</v>
+      </c>
+      <c r="C6" s="35">
+        <v>1</v>
       </c>
       <c r="D6" s="21">
-        <v>3956.71</v>
+        <v>1886</v>
       </c>
       <c r="E6" s="21">
-        <v>3885.55</v>
+        <v>1850</v>
       </c>
       <c r="F6" s="21">
-        <v>71.16</v>
+        <v>36</v>
       </c>
       <c r="G6" s="21">
-        <v>1.48</v>
+        <v>0.93</v>
       </c>
       <c r="H6" s="21">
         <v>8.22</v>
       </c>
-      <c r="I6" s="31">
-        <v>61.46</v>
+      <c r="I6" s="30">
+        <v>26.85</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -4140,9 +3567,9 @@
         <v>7</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>170</v>
-      </c>
-      <c r="C7" s="37">
+        <v>154</v>
+      </c>
+      <c r="C7" s="36">
         <v>1</v>
       </c>
       <c r="D7" s="27">
@@ -4160,7 +3587,7 @@
       <c r="H7" s="27">
         <v>0</v>
       </c>
-      <c r="I7" s="34">
+      <c r="I7" s="33">
         <v>2</v>
       </c>
     </row>
@@ -4199,7 +3626,7 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>171</v>
+        <v>155</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4225,7 +3652,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>172</v>
+        <v>156</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -4238,7 +3665,7 @@
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>173</v>
+        <v>157</v>
       </c>
       <c r="B5" s="15" t="s">
         <v>49</v>
@@ -4256,13 +3683,13 @@
         <v>57</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>174</v>
+        <v>158</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>175</v>
+        <v>159</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>176</v>
+        <v>160</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -4291,7 +3718,7 @@
         <v>0.925</v>
       </c>
       <c r="I6" s="17" t="s">
-        <v>177</v>
+        <v>161</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -4320,23 +3747,23 @@
         <v>0.55725</v>
       </c>
       <c r="I7" s="23" t="s">
-        <v>177</v>
+        <v>161</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="38" t="s">
-        <v>178</v>
-      </c>
-      <c r="H9" s="39">
+      <c r="A9" s="37" t="s">
+        <v>162</v>
+      </c>
+      <c r="H9" s="38">
         <f>SUMIFS(H6:H7,D6:D7,"USDT/PEN")</f>
         <v>1.48225</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="38" t="s">
-        <v>179</v>
-      </c>
-      <c r="H10" s="39">
+      <c r="A10" s="37" t="s">
+        <v>163</v>
+      </c>
+      <c r="H10" s="38">
         <f>SUMIFS(H6:H7,D6:D7,"USDT/USD")</f>
         <v>0</v>
       </c>
@@ -4376,7 +3803,7 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>180</v>
+        <v>164</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4402,7 +3829,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>181</v>
+        <v>165</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -4415,31 +3842,31 @@
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
-        <v>173</v>
+        <v>157</v>
       </c>
       <c r="B5" s="15" t="s">
         <v>53</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>182</v>
+        <v>166</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>49</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>183</v>
+        <v>167</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>174</v>
+        <v>158</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>175</v>
+        <v>159</v>
       </c>
       <c r="H5" s="15" t="s">
         <v>61</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>184</v>
+        <v>168</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -4450,7 +3877,7 @@
         <v>6</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>185</v>
+        <v>169</v>
       </c>
       <c r="D6" s="17" t="s">
         <v>68</v>
@@ -4479,7 +3906,7 @@
         <v>6</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>186</v>
+        <v>170</v>
       </c>
       <c r="D7" s="23" t="s">
         <v>75</v>
@@ -4488,7 +3915,7 @@
         <v>4.5</v>
       </c>
       <c r="F7" s="23" t="s">
-        <v>158</v>
+        <v>142</v>
       </c>
       <c r="G7" s="27">
         <v>4.5</v>

</xml_diff>